<commit_message>
The tendonlength graph was taken
</commit_message>
<xml_diff>
--- a/OpenSim practicle/gait.xlsx
+++ b/OpenSim practicle/gait.xlsx
@@ -8,12 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Ideas\Biomechanics\OpenSim practicle\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A763557B-A25C-48C2-9E82-E0AE04BBB2FC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{958AF4DF-B601-4714-B69D-547ECEE03B56}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Knee angle" sheetId="1" r:id="rId1"/>
+    <sheet name="Muscle Tendon Length" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -25,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="4">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="6">
   <si>
     <t>time</t>
   </si>
@@ -37,6 +38,12 @@
   </si>
   <si>
     <t>crouch1_gait</t>
+  </si>
+  <si>
+    <t>semiten_r</t>
+  </si>
+  <si>
+    <t>Normal gait</t>
   </si>
 </sst>
 </file>
@@ -166,7 +173,7 @@
               <a:cs typeface="+mn-cs"/>
             </a:defRPr>
           </a:pPr>
-          <a:endParaRPr lang="en-US"/>
+          <a:endParaRPr lang="en-GB"/>
         </a:p>
       </c:txPr>
     </c:title>
@@ -1618,6 +1625,1475 @@
 </c:chartSpace>
 </file>
 
+<file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="en-US"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:chart>
+    <c:autoTitleDeleted val="1"/>
+    <c:plotArea>
+      <c:layout>
+        <c:manualLayout>
+          <c:layoutTarget val="inner"/>
+          <c:xMode val="edge"/>
+          <c:yMode val="edge"/>
+          <c:x val="0.14445603674540683"/>
+          <c:y val="5.0925925925925923E-2"/>
+          <c:w val="0.65815463692038501"/>
+          <c:h val="0.74350320793234181"/>
+        </c:manualLayout>
+      </c:layout>
+      <c:scatterChart>
+        <c:scatterStyle val="smoothMarker"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:v>Normal Gait</c:v>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="19050" cap="rnd">
+              <a:solidFill>
+                <a:schemeClr val="accent1"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="none"/>
+          </c:marker>
+          <c:xVal>
+            <c:numRef>
+              <c:f>'Muscle Tendon Length'!$B$2:$B$52</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="51"/>
+                <c:pt idx="0">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>0.02</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>0.04</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>0.06</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>0.08</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>0.1</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>0.12</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>0.14000000000000001</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>0.16</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>0.18</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>0.2</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>0.22</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>0.24</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>0.26</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>0.28000000000000003</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>0.3</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>0.32</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>0.34</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>0.36</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>0.38</c:v>
+                </c:pt>
+                <c:pt idx="20">
+                  <c:v>0.4</c:v>
+                </c:pt>
+                <c:pt idx="21">
+                  <c:v>0.42</c:v>
+                </c:pt>
+                <c:pt idx="22">
+                  <c:v>0.44</c:v>
+                </c:pt>
+                <c:pt idx="23">
+                  <c:v>0.46</c:v>
+                </c:pt>
+                <c:pt idx="24">
+                  <c:v>0.48</c:v>
+                </c:pt>
+                <c:pt idx="25">
+                  <c:v>0.5</c:v>
+                </c:pt>
+                <c:pt idx="26">
+                  <c:v>0.52</c:v>
+                </c:pt>
+                <c:pt idx="27">
+                  <c:v>0.54</c:v>
+                </c:pt>
+                <c:pt idx="28">
+                  <c:v>0.56000000000000005</c:v>
+                </c:pt>
+                <c:pt idx="29">
+                  <c:v>0.57999999999999996</c:v>
+                </c:pt>
+                <c:pt idx="30">
+                  <c:v>0.6</c:v>
+                </c:pt>
+                <c:pt idx="31">
+                  <c:v>0.62</c:v>
+                </c:pt>
+                <c:pt idx="32">
+                  <c:v>0.64</c:v>
+                </c:pt>
+                <c:pt idx="33">
+                  <c:v>0.66</c:v>
+                </c:pt>
+                <c:pt idx="34">
+                  <c:v>0.68</c:v>
+                </c:pt>
+                <c:pt idx="35">
+                  <c:v>0.7</c:v>
+                </c:pt>
+                <c:pt idx="36">
+                  <c:v>0.72</c:v>
+                </c:pt>
+                <c:pt idx="37">
+                  <c:v>0.74</c:v>
+                </c:pt>
+                <c:pt idx="38">
+                  <c:v>0.76</c:v>
+                </c:pt>
+                <c:pt idx="39">
+                  <c:v>0.78</c:v>
+                </c:pt>
+                <c:pt idx="40">
+                  <c:v>0.8</c:v>
+                </c:pt>
+                <c:pt idx="41">
+                  <c:v>0.82</c:v>
+                </c:pt>
+                <c:pt idx="42">
+                  <c:v>0.84</c:v>
+                </c:pt>
+                <c:pt idx="43">
+                  <c:v>0.86</c:v>
+                </c:pt>
+                <c:pt idx="44">
+                  <c:v>0.88</c:v>
+                </c:pt>
+                <c:pt idx="45">
+                  <c:v>0.9</c:v>
+                </c:pt>
+                <c:pt idx="46">
+                  <c:v>0.92</c:v>
+                </c:pt>
+                <c:pt idx="47">
+                  <c:v>0.94</c:v>
+                </c:pt>
+                <c:pt idx="48">
+                  <c:v>0.96</c:v>
+                </c:pt>
+                <c:pt idx="49">
+                  <c:v>0.98</c:v>
+                </c:pt>
+                <c:pt idx="50">
+                  <c:v>1</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>'Muscle Tendon Length'!$C$2:$C$52</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="51"/>
+                <c:pt idx="0">
+                  <c:v>0.48773908999999999</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>0.48538869000000001</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>0.48270436999999999</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>0.47977209999999998</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>0.47669737000000001</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>0.47376028999999997</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>0.47118123000000001</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>0.46896335</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>0.46706026</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>0.46537708</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>0.46380811999999999</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>0.46234762000000001</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>0.46098807000000003</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>0.45970333000000002</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>0.45846753000000001</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>0.45727046999999998</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>0.45607057000000001</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>0.45486665999999998</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>0.45362539000000002</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>0.45233266</c:v>
+                </c:pt>
+                <c:pt idx="20">
+                  <c:v>0.45095113999999997</c:v>
+                </c:pt>
+                <c:pt idx="21">
+                  <c:v>0.44947178999999998</c:v>
+                </c:pt>
+                <c:pt idx="22">
+                  <c:v>0.44789551</c:v>
+                </c:pt>
+                <c:pt idx="23">
+                  <c:v>0.44624704999999998</c:v>
+                </c:pt>
+                <c:pt idx="24">
+                  <c:v>0.44444370999999999</c:v>
+                </c:pt>
+                <c:pt idx="25">
+                  <c:v>0.44250952999999998</c:v>
+                </c:pt>
+                <c:pt idx="26">
+                  <c:v>0.44038599</c:v>
+                </c:pt>
+                <c:pt idx="27">
+                  <c:v>0.43808888000000001</c:v>
+                </c:pt>
+                <c:pt idx="28">
+                  <c:v>0.43564523999999999</c:v>
+                </c:pt>
+                <c:pt idx="29">
+                  <c:v>0.43316806000000002</c:v>
+                </c:pt>
+                <c:pt idx="30">
+                  <c:v>0.43062085</c:v>
+                </c:pt>
+                <c:pt idx="31">
+                  <c:v>0.42825240999999997</c:v>
+                </c:pt>
+                <c:pt idx="32">
+                  <c:v>0.4265195</c:v>
+                </c:pt>
+                <c:pt idx="33">
+                  <c:v>0.42578650000000001</c:v>
+                </c:pt>
+                <c:pt idx="34">
+                  <c:v>0.42630374999999998</c:v>
+                </c:pt>
+                <c:pt idx="35">
+                  <c:v>0.42816236000000002</c:v>
+                </c:pt>
+                <c:pt idx="36">
+                  <c:v>0.43120671999999999</c:v>
+                </c:pt>
+                <c:pt idx="37">
+                  <c:v>0.43515010999999998</c:v>
+                </c:pt>
+                <c:pt idx="38">
+                  <c:v>0.43985079999999999</c:v>
+                </c:pt>
+                <c:pt idx="39">
+                  <c:v>0.44524525999999998</c:v>
+                </c:pt>
+                <c:pt idx="40">
+                  <c:v>0.45118132</c:v>
+                </c:pt>
+                <c:pt idx="41">
+                  <c:v>0.45747492000000001</c:v>
+                </c:pt>
+                <c:pt idx="42">
+                  <c:v>0.46395199999999998</c:v>
+                </c:pt>
+                <c:pt idx="43">
+                  <c:v>0.47029625000000003</c:v>
+                </c:pt>
+                <c:pt idx="44">
+                  <c:v>0.4761572</c:v>
+                </c:pt>
+                <c:pt idx="45">
+                  <c:v>0.48118638000000002</c:v>
+                </c:pt>
+                <c:pt idx="46">
+                  <c:v>0.48525578000000003</c:v>
+                </c:pt>
+                <c:pt idx="47">
+                  <c:v>0.48792676000000001</c:v>
+                </c:pt>
+                <c:pt idx="48">
+                  <c:v>0.48913962</c:v>
+                </c:pt>
+                <c:pt idx="49">
+                  <c:v>0.48900544000000001</c:v>
+                </c:pt>
+                <c:pt idx="50">
+                  <c:v>0.48766811999999998</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:yVal>
+          <c:smooth val="1"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-2A7C-498A-8128-C41935CE3115}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="1"/>
+          <c:order val="1"/>
+          <c:tx>
+            <c:v>Crouch Gait</c:v>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="19050" cap="rnd">
+              <a:solidFill>
+                <a:schemeClr val="accent2"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="none"/>
+          </c:marker>
+          <c:xVal>
+            <c:numRef>
+              <c:f>'Muscle Tendon Length'!$F$2:$F$120</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="119"/>
+                <c:pt idx="0">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>8.4745700000000007E-3</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>1.694915E-2</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>2.5423729999999999E-2</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>3.3898299999999999E-2</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>4.237287E-2</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>5.0847450000000002E-2</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>5.9322029999999998E-2</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>6.7796599999999999E-2</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>7.6271169999999999E-2</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>8.4745749999999995E-2</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>9.3220330000000004E-2</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>0.1016949</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>0.11016948</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>0.11864405</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>0.12711863000000001</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>0.1355932</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>0.14406778000000001</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>0.15254234999999999</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>0.16101693</c:v>
+                </c:pt>
+                <c:pt idx="20">
+                  <c:v>0.16949149999999999</c:v>
+                </c:pt>
+                <c:pt idx="21">
+                  <c:v>0.17796608</c:v>
+                </c:pt>
+                <c:pt idx="22">
+                  <c:v>0.18644065000000001</c:v>
+                </c:pt>
+                <c:pt idx="23">
+                  <c:v>0.19491522</c:v>
+                </c:pt>
+                <c:pt idx="24">
+                  <c:v>0.20338980000000001</c:v>
+                </c:pt>
+                <c:pt idx="25">
+                  <c:v>0.21186437</c:v>
+                </c:pt>
+                <c:pt idx="26">
+                  <c:v>0.22033895000000001</c:v>
+                </c:pt>
+                <c:pt idx="27">
+                  <c:v>0.22881351999999999</c:v>
+                </c:pt>
+                <c:pt idx="28">
+                  <c:v>0.2372881</c:v>
+                </c:pt>
+                <c:pt idx="29">
+                  <c:v>0.24576268000000001</c:v>
+                </c:pt>
+                <c:pt idx="30">
+                  <c:v>0.25423725000000003</c:v>
+                </c:pt>
+                <c:pt idx="31">
+                  <c:v>0.26271182999999998</c:v>
+                </c:pt>
+                <c:pt idx="32">
+                  <c:v>0.27118639999999999</c:v>
+                </c:pt>
+                <c:pt idx="33">
+                  <c:v>0.27966097000000001</c:v>
+                </c:pt>
+                <c:pt idx="34">
+                  <c:v>0.28813555000000002</c:v>
+                </c:pt>
+                <c:pt idx="35">
+                  <c:v>0.29661013000000003</c:v>
+                </c:pt>
+                <c:pt idx="36">
+                  <c:v>0.30508469999999999</c:v>
+                </c:pt>
+                <c:pt idx="37">
+                  <c:v>0.31355928</c:v>
+                </c:pt>
+                <c:pt idx="38">
+                  <c:v>0.32203385000000001</c:v>
+                </c:pt>
+                <c:pt idx="39">
+                  <c:v>0.33050842000000002</c:v>
+                </c:pt>
+                <c:pt idx="40">
+                  <c:v>0.33898299999999998</c:v>
+                </c:pt>
+                <c:pt idx="41">
+                  <c:v>0.34745757999999999</c:v>
+                </c:pt>
+                <c:pt idx="42">
+                  <c:v>0.35593215</c:v>
+                </c:pt>
+                <c:pt idx="43">
+                  <c:v>0.36440672000000002</c:v>
+                </c:pt>
+                <c:pt idx="44">
+                  <c:v>0.37288130000000003</c:v>
+                </c:pt>
+                <c:pt idx="45">
+                  <c:v>0.38135587999999998</c:v>
+                </c:pt>
+                <c:pt idx="46">
+                  <c:v>0.38983045</c:v>
+                </c:pt>
+                <c:pt idx="47">
+                  <c:v>0.39830502000000001</c:v>
+                </c:pt>
+                <c:pt idx="48">
+                  <c:v>0.40677960000000002</c:v>
+                </c:pt>
+                <c:pt idx="49">
+                  <c:v>0.41525417999999997</c:v>
+                </c:pt>
+                <c:pt idx="50">
+                  <c:v>0.42372874999999999</c:v>
+                </c:pt>
+                <c:pt idx="51">
+                  <c:v>0.43220333</c:v>
+                </c:pt>
+                <c:pt idx="52">
+                  <c:v>0.44067790000000001</c:v>
+                </c:pt>
+                <c:pt idx="53">
+                  <c:v>0.44915247000000003</c:v>
+                </c:pt>
+                <c:pt idx="54">
+                  <c:v>0.45762704999999998</c:v>
+                </c:pt>
+                <c:pt idx="55">
+                  <c:v>0.46610162999999999</c:v>
+                </c:pt>
+                <c:pt idx="56">
+                  <c:v>0.4745762</c:v>
+                </c:pt>
+                <c:pt idx="57">
+                  <c:v>0.48305077000000002</c:v>
+                </c:pt>
+                <c:pt idx="58">
+                  <c:v>0.49152535000000003</c:v>
+                </c:pt>
+                <c:pt idx="59">
+                  <c:v>0.49999992999999998</c:v>
+                </c:pt>
+                <c:pt idx="60">
+                  <c:v>0.50847450000000005</c:v>
+                </c:pt>
+                <c:pt idx="61">
+                  <c:v>0.51694907000000001</c:v>
+                </c:pt>
+                <c:pt idx="62">
+                  <c:v>0.52542365000000002</c:v>
+                </c:pt>
+                <c:pt idx="63">
+                  <c:v>0.53389821999999998</c:v>
+                </c:pt>
+                <c:pt idx="64">
+                  <c:v>0.54237279999999999</c:v>
+                </c:pt>
+                <c:pt idx="65">
+                  <c:v>0.55084738</c:v>
+                </c:pt>
+                <c:pt idx="66">
+                  <c:v>0.55932194999999996</c:v>
+                </c:pt>
+                <c:pt idx="67">
+                  <c:v>0.56779652000000003</c:v>
+                </c:pt>
+                <c:pt idx="68">
+                  <c:v>0.57627110000000004</c:v>
+                </c:pt>
+                <c:pt idx="69">
+                  <c:v>0.58474567</c:v>
+                </c:pt>
+                <c:pt idx="70">
+                  <c:v>0.59322025</c:v>
+                </c:pt>
+                <c:pt idx="71">
+                  <c:v>0.60169483000000001</c:v>
+                </c:pt>
+                <c:pt idx="72">
+                  <c:v>0.61016939999999997</c:v>
+                </c:pt>
+                <c:pt idx="73">
+                  <c:v>0.61864397999999998</c:v>
+                </c:pt>
+                <c:pt idx="74">
+                  <c:v>0.62711855000000005</c:v>
+                </c:pt>
+                <c:pt idx="75">
+                  <c:v>0.63559312000000001</c:v>
+                </c:pt>
+                <c:pt idx="76">
+                  <c:v>0.64406770000000002</c:v>
+                </c:pt>
+                <c:pt idx="77">
+                  <c:v>0.65254226999999998</c:v>
+                </c:pt>
+                <c:pt idx="78">
+                  <c:v>0.66101684999999999</c:v>
+                </c:pt>
+                <c:pt idx="79">
+                  <c:v>0.66949143</c:v>
+                </c:pt>
+                <c:pt idx="80">
+                  <c:v>0.67796599999999996</c:v>
+                </c:pt>
+                <c:pt idx="81">
+                  <c:v>0.68644057000000003</c:v>
+                </c:pt>
+                <c:pt idx="82">
+                  <c:v>0.69491515000000004</c:v>
+                </c:pt>
+                <c:pt idx="83">
+                  <c:v>0.70338972</c:v>
+                </c:pt>
+                <c:pt idx="84">
+                  <c:v>0.71186430000000001</c:v>
+                </c:pt>
+                <c:pt idx="85">
+                  <c:v>0.72033888000000001</c:v>
+                </c:pt>
+                <c:pt idx="86">
+                  <c:v>0.72881344999999997</c:v>
+                </c:pt>
+                <c:pt idx="87">
+                  <c:v>0.73728802999999998</c:v>
+                </c:pt>
+                <c:pt idx="88">
+                  <c:v>0.74576260000000005</c:v>
+                </c:pt>
+                <c:pt idx="89">
+                  <c:v>0.75423717000000001</c:v>
+                </c:pt>
+                <c:pt idx="90">
+                  <c:v>0.76271175000000002</c:v>
+                </c:pt>
+                <c:pt idx="91">
+                  <c:v>0.77118631999999998</c:v>
+                </c:pt>
+                <c:pt idx="92">
+                  <c:v>0.77966089999999999</c:v>
+                </c:pt>
+                <c:pt idx="93">
+                  <c:v>0.78813548</c:v>
+                </c:pt>
+                <c:pt idx="94">
+                  <c:v>0.79661004999999996</c:v>
+                </c:pt>
+                <c:pt idx="95">
+                  <c:v>0.80508462000000003</c:v>
+                </c:pt>
+                <c:pt idx="96">
+                  <c:v>0.81355920000000004</c:v>
+                </c:pt>
+                <c:pt idx="97">
+                  <c:v>0.82203377</c:v>
+                </c:pt>
+                <c:pt idx="98">
+                  <c:v>0.83050835000000001</c:v>
+                </c:pt>
+                <c:pt idx="99">
+                  <c:v>0.83898293000000002</c:v>
+                </c:pt>
+                <c:pt idx="100">
+                  <c:v>0.84745749999999997</c:v>
+                </c:pt>
+                <c:pt idx="101">
+                  <c:v>0.85593207999999998</c:v>
+                </c:pt>
+                <c:pt idx="102">
+                  <c:v>0.86440665000000005</c:v>
+                </c:pt>
+                <c:pt idx="103">
+                  <c:v>0.87288122000000001</c:v>
+                </c:pt>
+                <c:pt idx="104">
+                  <c:v>0.88135580000000002</c:v>
+                </c:pt>
+                <c:pt idx="105">
+                  <c:v>0.88983036999999998</c:v>
+                </c:pt>
+                <c:pt idx="106">
+                  <c:v>0.89830494999999999</c:v>
+                </c:pt>
+                <c:pt idx="107">
+                  <c:v>0.90677953</c:v>
+                </c:pt>
+                <c:pt idx="108">
+                  <c:v>0.91525409999999996</c:v>
+                </c:pt>
+                <c:pt idx="109">
+                  <c:v>0.92372867000000003</c:v>
+                </c:pt>
+                <c:pt idx="110">
+                  <c:v>0.93220325000000004</c:v>
+                </c:pt>
+                <c:pt idx="111">
+                  <c:v>0.94067782</c:v>
+                </c:pt>
+                <c:pt idx="112">
+                  <c:v>0.94915240000000001</c:v>
+                </c:pt>
+                <c:pt idx="113">
+                  <c:v>0.95762698000000002</c:v>
+                </c:pt>
+                <c:pt idx="114">
+                  <c:v>0.96610154999999998</c:v>
+                </c:pt>
+                <c:pt idx="115">
+                  <c:v>0.97457612999999998</c:v>
+                </c:pt>
+                <c:pt idx="116">
+                  <c:v>0.98305070000000006</c:v>
+                </c:pt>
+                <c:pt idx="117">
+                  <c:v>0.99152534999999997</c:v>
+                </c:pt>
+                <c:pt idx="118">
+                  <c:v>1</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>'Muscle Tendon Length'!$G$2:$G$120</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="119"/>
+                <c:pt idx="0">
+                  <c:v>0.47530866999999999</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>0.47406695999999998</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>0.47282750000000001</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>0.4717905</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>0.47075814999999999</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>0.47007483999999999</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>0.46939413000000002</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>0.46901558999999998</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>0.46863789</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>0.46848369000000001</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>0.46832971000000001</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>0.46830638000000002</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>0.46828288000000001</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>0.46829394000000002</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>0.46830503000000001</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>0.46831993999999999</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>0.46833511</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>0.46829721000000002</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>0.46825948000000001</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>0.46801118000000003</c:v>
+                </c:pt>
+                <c:pt idx="20">
+                  <c:v>0.46776284000000001</c:v>
+                </c:pt>
+                <c:pt idx="21">
+                  <c:v>0.46725118999999998</c:v>
+                </c:pt>
+                <c:pt idx="22">
+                  <c:v>0.46673947999999998</c:v>
+                </c:pt>
+                <c:pt idx="23">
+                  <c:v>0.46597948</c:v>
+                </c:pt>
+                <c:pt idx="24">
+                  <c:v>0.46521911999999999</c:v>
+                </c:pt>
+                <c:pt idx="25">
+                  <c:v>0.46422855000000002</c:v>
+                </c:pt>
+                <c:pt idx="26">
+                  <c:v>0.46323663999999998</c:v>
+                </c:pt>
+                <c:pt idx="27">
+                  <c:v>0.46196310000000002</c:v>
+                </c:pt>
+                <c:pt idx="28">
+                  <c:v>0.46068764000000001</c:v>
+                </c:pt>
+                <c:pt idx="29">
+                  <c:v>0.45908892000000001</c:v>
+                </c:pt>
+                <c:pt idx="30">
+                  <c:v>0.45748892000000002</c:v>
+                </c:pt>
+                <c:pt idx="31">
+                  <c:v>0.45574121000000001</c:v>
+                </c:pt>
+                <c:pt idx="32">
+                  <c:v>0.45399355000000002</c:v>
+                </c:pt>
+                <c:pt idx="33">
+                  <c:v>0.45232782999999999</c:v>
+                </c:pt>
+                <c:pt idx="34">
+                  <c:v>0.45066324000000002</c:v>
+                </c:pt>
+                <c:pt idx="35">
+                  <c:v>0.44916756000000002</c:v>
+                </c:pt>
+                <c:pt idx="36">
+                  <c:v>0.44767460999999997</c:v>
+                </c:pt>
+                <c:pt idx="37">
+                  <c:v>0.44623963999999999</c:v>
+                </c:pt>
+                <c:pt idx="38">
+                  <c:v>0.44480872999999999</c:v>
+                </c:pt>
+                <c:pt idx="39">
+                  <c:v>0.44334434</c:v>
+                </c:pt>
+                <c:pt idx="40">
+                  <c:v>0.44188388000000001</c:v>
+                </c:pt>
+                <c:pt idx="41">
+                  <c:v>0.44044678999999998</c:v>
+                </c:pt>
+                <c:pt idx="42">
+                  <c:v>0.43901251000000002</c:v>
+                </c:pt>
+                <c:pt idx="43">
+                  <c:v>0.43771446000000003</c:v>
+                </c:pt>
+                <c:pt idx="44">
+                  <c:v>0.43641889</c:v>
+                </c:pt>
+                <c:pt idx="45">
+                  <c:v>0.43539305</c:v>
+                </c:pt>
+                <c:pt idx="46">
+                  <c:v>0.43436929000000002</c:v>
+                </c:pt>
+                <c:pt idx="47">
+                  <c:v>0.43362592999999999</c:v>
+                </c:pt>
+                <c:pt idx="48">
+                  <c:v>0.43288390999999998</c:v>
+                </c:pt>
+                <c:pt idx="49">
+                  <c:v>0.43222160999999998</c:v>
+                </c:pt>
+                <c:pt idx="50">
+                  <c:v>0.43155992999999998</c:v>
+                </c:pt>
+                <c:pt idx="51">
+                  <c:v>0.43091254000000001</c:v>
+                </c:pt>
+                <c:pt idx="52">
+                  <c:v>0.43026740000000002</c:v>
+                </c:pt>
+                <c:pt idx="53">
+                  <c:v>0.42978358</c:v>
+                </c:pt>
+                <c:pt idx="54">
+                  <c:v>0.42930288999999999</c:v>
+                </c:pt>
+                <c:pt idx="55">
+                  <c:v>0.42906586000000002</c:v>
+                </c:pt>
+                <c:pt idx="56">
+                  <c:v>0.42882979999999998</c:v>
+                </c:pt>
+                <c:pt idx="57">
+                  <c:v>0.42864949000000002</c:v>
+                </c:pt>
+                <c:pt idx="58">
+                  <c:v>0.42846964999999998</c:v>
+                </c:pt>
+                <c:pt idx="59">
+                  <c:v>0.42820206999999999</c:v>
+                </c:pt>
+                <c:pt idx="60">
+                  <c:v>0.42793581000000003</c:v>
+                </c:pt>
+                <c:pt idx="61">
+                  <c:v>0.42771532000000001</c:v>
+                </c:pt>
+                <c:pt idx="62">
+                  <c:v>0.42749680000000001</c:v>
+                </c:pt>
+                <c:pt idx="63">
+                  <c:v>0.42745514000000001</c:v>
+                </c:pt>
+                <c:pt idx="64">
+                  <c:v>0.42741535000000003</c:v>
+                </c:pt>
+                <c:pt idx="65">
+                  <c:v>0.42759623000000002</c:v>
+                </c:pt>
+                <c:pt idx="66">
+                  <c:v>0.42777897999999998</c:v>
+                </c:pt>
+                <c:pt idx="67">
+                  <c:v>0.42811188999999999</c:v>
+                </c:pt>
+                <c:pt idx="68">
+                  <c:v>0.42844613999999998</c:v>
+                </c:pt>
+                <c:pt idx="69">
+                  <c:v>0.42887331000000001</c:v>
+                </c:pt>
+                <c:pt idx="70">
+                  <c:v>0.42930146000000002</c:v>
+                </c:pt>
+                <c:pt idx="71">
+                  <c:v>0.42975590000000002</c:v>
+                </c:pt>
+                <c:pt idx="72">
+                  <c:v>0.43021253999999998</c:v>
+                </c:pt>
+                <c:pt idx="73">
+                  <c:v>0.43070751000000002</c:v>
+                </c:pt>
+                <c:pt idx="74">
+                  <c:v>0.43120595</c:v>
+                </c:pt>
+                <c:pt idx="75">
+                  <c:v>0.43181671999999999</c:v>
+                </c:pt>
+                <c:pt idx="76">
+                  <c:v>0.43243105999999998</c:v>
+                </c:pt>
+                <c:pt idx="77">
+                  <c:v>0.43321780999999998</c:v>
+                </c:pt>
+                <c:pt idx="78">
+                  <c:v>0.43400782999999998</c:v>
+                </c:pt>
+                <c:pt idx="79">
+                  <c:v>0.43502440999999997</c:v>
+                </c:pt>
+                <c:pt idx="80">
+                  <c:v>0.43604457000000002</c:v>
+                </c:pt>
+                <c:pt idx="81">
+                  <c:v>0.43732399</c:v>
+                </c:pt>
+                <c:pt idx="82">
+                  <c:v>0.43860950999999998</c:v>
+                </c:pt>
+                <c:pt idx="83">
+                  <c:v>0.44013275000000002</c:v>
+                </c:pt>
+                <c:pt idx="84">
+                  <c:v>0.44166603999999998</c:v>
+                </c:pt>
+                <c:pt idx="85">
+                  <c:v>0.44328474000000001</c:v>
+                </c:pt>
+                <c:pt idx="86">
+                  <c:v>0.44491585</c:v>
+                </c:pt>
+                <c:pt idx="87">
+                  <c:v>0.44649826999999997</c:v>
+                </c:pt>
+                <c:pt idx="88">
+                  <c:v>0.44809381999999998</c:v>
+                </c:pt>
+                <c:pt idx="89">
+                  <c:v>0.44960991</c:v>
+                </c:pt>
+                <c:pt idx="90">
+                  <c:v>0.45113906999999998</c:v>
+                </c:pt>
+                <c:pt idx="91">
+                  <c:v>0.45259044999999998</c:v>
+                </c:pt>
+                <c:pt idx="92">
+                  <c:v>0.45405624</c:v>
+                </c:pt>
+                <c:pt idx="93">
+                  <c:v>0.45540003000000001</c:v>
+                </c:pt>
+                <c:pt idx="94">
+                  <c:v>0.45676240000000001</c:v>
+                </c:pt>
+                <c:pt idx="95">
+                  <c:v>0.45801246000000001</c:v>
+                </c:pt>
+                <c:pt idx="96">
+                  <c:v>0.45928313999999998</c:v>
+                </c:pt>
+                <c:pt idx="97">
+                  <c:v>0.46052575000000001</c:v>
+                </c:pt>
+                <c:pt idx="98">
+                  <c:v>0.46178088</c:v>
+                </c:pt>
+                <c:pt idx="99">
+                  <c:v>0.46308433999999998</c:v>
+                </c:pt>
+                <c:pt idx="100">
+                  <c:v>0.46438994</c:v>
+                </c:pt>
+                <c:pt idx="101">
+                  <c:v>0.46582235999999999</c:v>
+                </c:pt>
+                <c:pt idx="102">
+                  <c:v>0.46725633</c:v>
+                </c:pt>
+                <c:pt idx="103">
+                  <c:v>0.46882960000000001</c:v>
+                </c:pt>
+                <c:pt idx="104">
+                  <c:v>0.47040977</c:v>
+                </c:pt>
+                <c:pt idx="105">
+                  <c:v>0.47194008999999998</c:v>
+                </c:pt>
+                <c:pt idx="106">
+                  <c:v>0.47348068999999998</c:v>
+                </c:pt>
+                <c:pt idx="107">
+                  <c:v>0.47464234</c:v>
+                </c:pt>
+                <c:pt idx="108">
+                  <c:v>0.47581240000000002</c:v>
+                </c:pt>
+                <c:pt idx="109">
+                  <c:v>0.47638794000000001</c:v>
+                </c:pt>
+                <c:pt idx="110">
+                  <c:v>0.47696629000000001</c:v>
+                </c:pt>
+                <c:pt idx="111">
+                  <c:v>0.47702480000000003</c:v>
+                </c:pt>
+                <c:pt idx="112">
+                  <c:v>0.47708181999999999</c:v>
+                </c:pt>
+                <c:pt idx="113">
+                  <c:v>0.47682298000000001</c:v>
+                </c:pt>
+                <c:pt idx="114">
+                  <c:v>0.47656331000000002</c:v>
+                </c:pt>
+                <c:pt idx="115">
+                  <c:v>0.47612222999999998</c:v>
+                </c:pt>
+                <c:pt idx="116">
+                  <c:v>0.47568112000000001</c:v>
+                </c:pt>
+                <c:pt idx="117">
+                  <c:v>0.47500200999999997</c:v>
+                </c:pt>
+                <c:pt idx="118">
+                  <c:v>0.47432417999999998</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:yVal>
+          <c:smooth val="1"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000001-2A7C-498A-8128-C41935CE3115}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:axId val="839426752"/>
+        <c:axId val="646647648"/>
+      </c:scatterChart>
+      <c:valAx>
+        <c:axId val="839426752"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="tx1">
+                        <a:lumMod val="65000"/>
+                        <a:lumOff val="35000"/>
+                      </a:schemeClr>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:rPr lang="en-GB"/>
+                  <a:t>Gait Cycle</a:t>
+                </a:r>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:overlay val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1">
+                      <a:lumMod val="65000"/>
+                      <a:lumOff val="35000"/>
+                    </a:schemeClr>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="en-US"/>
+            </a:p>
+          </c:txPr>
+        </c:title>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="25000"/>
+                <a:lumOff val="75000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="646647648"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="midCat"/>
+      </c:valAx>
+      <c:valAx>
+        <c:axId val="646647648"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr rot="-5400000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="tx1">
+                        <a:lumMod val="65000"/>
+                        <a:lumOff val="35000"/>
+                      </a:schemeClr>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:rPr lang="en-GB"/>
+                  <a:t>semite_r</a:t>
+                </a:r>
+                <a:r>
+                  <a:rPr lang="en-GB" baseline="0"/>
+                  <a:t> length</a:t>
+                </a:r>
+                <a:endParaRPr lang="en-GB"/>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:overlay val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="-5400000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1">
+                      <a:lumMod val="65000"/>
+                      <a:lumOff val="35000"/>
+                    </a:schemeClr>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="en-US"/>
+            </a:p>
+          </c:txPr>
+        </c:title>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="25000"/>
+                <a:lumOff val="75000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="839426752"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="midCat"/>
+      </c:valAx>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+    </c:plotArea>
+    <c:legend>
+      <c:legendPos val="r"/>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="en-US"/>
+        </a:p>
+      </c:txPr>
+    </c:legend>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
+    <c:extLst>
+      <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
+        <c16r3:dataDisplayOptions16>
+          <c16r3:dispNaAsBlank val="1"/>
+        </c16r3:dataDisplayOptions16>
+      </c:ext>
+    </c:extLst>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:schemeClr val="bg1"/>
+    </a:solidFill>
+    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:solidFill>
+        <a:schemeClr val="tx1">
+          <a:lumMod val="15000"/>
+          <a:lumOff val="85000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+    <a:effectLst/>
+  </c:spPr>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr/>
+      </a:pPr>
+      <a:endParaRPr lang="en-US"/>
+    </a:p>
+  </c:txPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
 <file path=xl/charts/colors1.xml><?xml version="1.0" encoding="utf-8"?>
 <cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
   <a:schemeClr val="accent1"/>
@@ -1658,7 +3134,563 @@
 </cs:colorStyle>
 </file>
 
+<file path=xl/charts/colors2.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
+  <a:schemeClr val="accent1"/>
+  <a:schemeClr val="accent2"/>
+  <a:schemeClr val="accent3"/>
+  <a:schemeClr val="accent4"/>
+  <a:schemeClr val="accent5"/>
+  <a:schemeClr val="accent6"/>
+  <cs:variation/>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+    <a:lumOff val="20000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+    <a:lumOff val="40000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+    <a:lumOff val="30000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+    <a:lumOff val="50000"/>
+  </cs:variation>
+</cs:colorStyle>
+</file>
+
 <file path=xl/charts/style1.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="240">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="bg1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="75000"/>
+          <a:lumOff val="25000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="5000"/>
+            <a:lumOff val="95000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="50000"/>
+            <a:lumOff val="50000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:legend>
+  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1400" b="0" kern="1200" spc="0" baseline="0"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:prstDash val="sysDot"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
+<file path=xl/charts/style2.xml><?xml version="1.0" encoding="utf-8"?>
 <cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="240">
   <cs:axisTitle>
     <cs:lnRef idx="0"/>
@@ -2494,6 +4526,47 @@
 </xdr:wsDr>
 </file>
 
+<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>495300</xdr:colOff>
+      <xdr:row>2</xdr:row>
+      <xdr:rowOff>171450</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>16</xdr:col>
+      <xdr:colOff>190500</xdr:colOff>
+      <xdr:row>17</xdr:row>
+      <xdr:rowOff>171450</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="2" name="Chart 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{D24B667D-8FBB-6A35-0D7E-F579C2063C98}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{A438BDB1-2506-4781-9134-0982BB3AFDAE}" name="Table1" displayName="Table1" ref="A1:C52" totalsRowShown="0" headerRowDxfId="0">
   <autoFilter ref="A1:C52" xr:uid="{A438BDB1-2506-4781-9134-0982BB3AFDAE}"/>
@@ -2515,6 +4588,30 @@
     <tableColumn id="3" xr3:uid="{FDAD7FE6-0A68-4FE9-9BA3-C12287F8CAE5}" name="knee_angle_r"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium14" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{DC38FC01-FC83-4A4D-BA8C-03BC92FED031}" name="Table3" displayName="Table3" ref="A1:C52" totalsRowShown="0">
+  <autoFilter ref="A1:C52" xr:uid="{DC38FC01-FC83-4A4D-BA8C-03BC92FED031}"/>
+  <tableColumns count="3">
+    <tableColumn id="1" xr3:uid="{541FE60D-BB00-4C6C-A1F7-07947B9A1689}" name="time"/>
+    <tableColumn id="2" xr3:uid="{4C775554-0428-44D8-82B3-930FE265FC3D}" name="normal_gait"/>
+    <tableColumn id="3" xr3:uid="{29F3F8E1-6F72-41E3-A408-64099A0BF26C}" name="Normal gait"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium14" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{720E6F7A-C1EE-498C-9E00-6C51B2EBB9ED}" name="Table4" displayName="Table4" ref="E1:G120" totalsRowShown="0">
+  <autoFilter ref="E1:G120" xr:uid="{720E6F7A-C1EE-498C-9E00-6C51B2EBB9ED}"/>
+  <tableColumns count="3">
+    <tableColumn id="1" xr3:uid="{EB5FBFFB-2FC5-4024-BFDC-89AD1D43F026}" name="time"/>
+    <tableColumn id="2" xr3:uid="{2EE4805D-D0EA-40A8-AD7C-EFC27C7B7F19}" name="crouch1_gait"/>
+    <tableColumn id="3" xr3:uid="{ECBEE375-0BD8-4D60-970B-0E6F88DB48B3}" name="semiten_r"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium7" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
@@ -4587,4 +6684,1814 @@
     <tablePart r:id="rId3"/>
   </tableParts>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A694D991-E7A4-4658-80A1-9E2FC06B3363}">
+  <dimension ref="A1:G120"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="6.5546875" customWidth="1"/>
+    <col min="2" max="2" width="12.6640625" customWidth="1"/>
+    <col min="3" max="3" width="12.44140625" customWidth="1"/>
+    <col min="6" max="6" width="13.44140625" customWidth="1"/>
+    <col min="7" max="7" width="11" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>5</v>
+      </c>
+      <c r="E1" t="s">
+        <v>0</v>
+      </c>
+      <c r="F1" t="s">
+        <v>3</v>
+      </c>
+      <c r="G1" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A2">
+        <v>0</v>
+      </c>
+      <c r="B2">
+        <v>0</v>
+      </c>
+      <c r="C2">
+        <v>0.48773908999999999</v>
+      </c>
+      <c r="E2">
+        <v>0</v>
+      </c>
+      <c r="F2">
+        <v>0</v>
+      </c>
+      <c r="G2">
+        <v>0.47530866999999999</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A3">
+        <v>1</v>
+      </c>
+      <c r="B3">
+        <v>0.02</v>
+      </c>
+      <c r="C3">
+        <v>0.48538869000000001</v>
+      </c>
+      <c r="E3">
+        <v>1</v>
+      </c>
+      <c r="F3">
+        <v>8.4745700000000007E-3</v>
+      </c>
+      <c r="G3">
+        <v>0.47406695999999998</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A4">
+        <v>2</v>
+      </c>
+      <c r="B4">
+        <v>0.04</v>
+      </c>
+      <c r="C4">
+        <v>0.48270436999999999</v>
+      </c>
+      <c r="E4">
+        <v>2</v>
+      </c>
+      <c r="F4">
+        <v>1.694915E-2</v>
+      </c>
+      <c r="G4">
+        <v>0.47282750000000001</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A5">
+        <v>3</v>
+      </c>
+      <c r="B5">
+        <v>0.06</v>
+      </c>
+      <c r="C5">
+        <v>0.47977209999999998</v>
+      </c>
+      <c r="E5">
+        <v>3</v>
+      </c>
+      <c r="F5">
+        <v>2.5423729999999999E-2</v>
+      </c>
+      <c r="G5">
+        <v>0.4717905</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A6">
+        <v>4</v>
+      </c>
+      <c r="B6">
+        <v>0.08</v>
+      </c>
+      <c r="C6">
+        <v>0.47669737000000001</v>
+      </c>
+      <c r="E6">
+        <v>4</v>
+      </c>
+      <c r="F6">
+        <v>3.3898299999999999E-2</v>
+      </c>
+      <c r="G6">
+        <v>0.47075814999999999</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A7">
+        <v>5</v>
+      </c>
+      <c r="B7">
+        <v>0.1</v>
+      </c>
+      <c r="C7">
+        <v>0.47376028999999997</v>
+      </c>
+      <c r="E7">
+        <v>5</v>
+      </c>
+      <c r="F7">
+        <v>4.237287E-2</v>
+      </c>
+      <c r="G7">
+        <v>0.47007483999999999</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A8">
+        <v>6</v>
+      </c>
+      <c r="B8">
+        <v>0.12</v>
+      </c>
+      <c r="C8">
+        <v>0.47118123000000001</v>
+      </c>
+      <c r="E8">
+        <v>6</v>
+      </c>
+      <c r="F8">
+        <v>5.0847450000000002E-2</v>
+      </c>
+      <c r="G8">
+        <v>0.46939413000000002</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A9">
+        <v>7</v>
+      </c>
+      <c r="B9">
+        <v>0.14000000000000001</v>
+      </c>
+      <c r="C9">
+        <v>0.46896335</v>
+      </c>
+      <c r="E9">
+        <v>7</v>
+      </c>
+      <c r="F9">
+        <v>5.9322029999999998E-2</v>
+      </c>
+      <c r="G9">
+        <v>0.46901558999999998</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A10">
+        <v>8</v>
+      </c>
+      <c r="B10">
+        <v>0.16</v>
+      </c>
+      <c r="C10">
+        <v>0.46706026</v>
+      </c>
+      <c r="E10">
+        <v>8</v>
+      </c>
+      <c r="F10">
+        <v>6.7796599999999999E-2</v>
+      </c>
+      <c r="G10">
+        <v>0.46863789</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A11">
+        <v>9</v>
+      </c>
+      <c r="B11">
+        <v>0.18</v>
+      </c>
+      <c r="C11">
+        <v>0.46537708</v>
+      </c>
+      <c r="E11">
+        <v>9</v>
+      </c>
+      <c r="F11">
+        <v>7.6271169999999999E-2</v>
+      </c>
+      <c r="G11">
+        <v>0.46848369000000001</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A12">
+        <v>10</v>
+      </c>
+      <c r="B12">
+        <v>0.2</v>
+      </c>
+      <c r="C12">
+        <v>0.46380811999999999</v>
+      </c>
+      <c r="E12">
+        <v>10</v>
+      </c>
+      <c r="F12">
+        <v>8.4745749999999995E-2</v>
+      </c>
+      <c r="G12">
+        <v>0.46832971000000001</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A13">
+        <v>11</v>
+      </c>
+      <c r="B13">
+        <v>0.22</v>
+      </c>
+      <c r="C13">
+        <v>0.46234762000000001</v>
+      </c>
+      <c r="E13">
+        <v>11</v>
+      </c>
+      <c r="F13">
+        <v>9.3220330000000004E-2</v>
+      </c>
+      <c r="G13">
+        <v>0.46830638000000002</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A14">
+        <v>12</v>
+      </c>
+      <c r="B14">
+        <v>0.24</v>
+      </c>
+      <c r="C14">
+        <v>0.46098807000000003</v>
+      </c>
+      <c r="E14">
+        <v>12</v>
+      </c>
+      <c r="F14">
+        <v>0.1016949</v>
+      </c>
+      <c r="G14">
+        <v>0.46828288000000001</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A15">
+        <v>13</v>
+      </c>
+      <c r="B15">
+        <v>0.26</v>
+      </c>
+      <c r="C15">
+        <v>0.45970333000000002</v>
+      </c>
+      <c r="E15">
+        <v>13</v>
+      </c>
+      <c r="F15">
+        <v>0.11016948</v>
+      </c>
+      <c r="G15">
+        <v>0.46829394000000002</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A16">
+        <v>14</v>
+      </c>
+      <c r="B16">
+        <v>0.28000000000000003</v>
+      </c>
+      <c r="C16">
+        <v>0.45846753000000001</v>
+      </c>
+      <c r="E16">
+        <v>14</v>
+      </c>
+      <c r="F16">
+        <v>0.11864405</v>
+      </c>
+      <c r="G16">
+        <v>0.46830503000000001</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A17">
+        <v>15</v>
+      </c>
+      <c r="B17">
+        <v>0.3</v>
+      </c>
+      <c r="C17">
+        <v>0.45727046999999998</v>
+      </c>
+      <c r="E17">
+        <v>15</v>
+      </c>
+      <c r="F17">
+        <v>0.12711863000000001</v>
+      </c>
+      <c r="G17">
+        <v>0.46831993999999999</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A18">
+        <v>16</v>
+      </c>
+      <c r="B18">
+        <v>0.32</v>
+      </c>
+      <c r="C18">
+        <v>0.45607057000000001</v>
+      </c>
+      <c r="E18">
+        <v>16</v>
+      </c>
+      <c r="F18">
+        <v>0.1355932</v>
+      </c>
+      <c r="G18">
+        <v>0.46833511</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A19">
+        <v>17</v>
+      </c>
+      <c r="B19">
+        <v>0.34</v>
+      </c>
+      <c r="C19">
+        <v>0.45486665999999998</v>
+      </c>
+      <c r="E19">
+        <v>17</v>
+      </c>
+      <c r="F19">
+        <v>0.14406778000000001</v>
+      </c>
+      <c r="G19">
+        <v>0.46829721000000002</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A20">
+        <v>18</v>
+      </c>
+      <c r="B20">
+        <v>0.36</v>
+      </c>
+      <c r="C20">
+        <v>0.45362539000000002</v>
+      </c>
+      <c r="E20">
+        <v>18</v>
+      </c>
+      <c r="F20">
+        <v>0.15254234999999999</v>
+      </c>
+      <c r="G20">
+        <v>0.46825948000000001</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A21">
+        <v>19</v>
+      </c>
+      <c r="B21">
+        <v>0.38</v>
+      </c>
+      <c r="C21">
+        <v>0.45233266</v>
+      </c>
+      <c r="E21">
+        <v>19</v>
+      </c>
+      <c r="F21">
+        <v>0.16101693</v>
+      </c>
+      <c r="G21">
+        <v>0.46801118000000003</v>
+      </c>
+    </row>
+    <row r="22" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A22">
+        <v>20</v>
+      </c>
+      <c r="B22">
+        <v>0.4</v>
+      </c>
+      <c r="C22">
+        <v>0.45095113999999997</v>
+      </c>
+      <c r="E22">
+        <v>20</v>
+      </c>
+      <c r="F22">
+        <v>0.16949149999999999</v>
+      </c>
+      <c r="G22">
+        <v>0.46776284000000001</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A23">
+        <v>21</v>
+      </c>
+      <c r="B23">
+        <v>0.42</v>
+      </c>
+      <c r="C23">
+        <v>0.44947178999999998</v>
+      </c>
+      <c r="E23">
+        <v>21</v>
+      </c>
+      <c r="F23">
+        <v>0.17796608</v>
+      </c>
+      <c r="G23">
+        <v>0.46725118999999998</v>
+      </c>
+    </row>
+    <row r="24" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A24">
+        <v>22</v>
+      </c>
+      <c r="B24">
+        <v>0.44</v>
+      </c>
+      <c r="C24">
+        <v>0.44789551</v>
+      </c>
+      <c r="E24">
+        <v>22</v>
+      </c>
+      <c r="F24">
+        <v>0.18644065000000001</v>
+      </c>
+      <c r="G24">
+        <v>0.46673947999999998</v>
+      </c>
+    </row>
+    <row r="25" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A25">
+        <v>23</v>
+      </c>
+      <c r="B25">
+        <v>0.46</v>
+      </c>
+      <c r="C25">
+        <v>0.44624704999999998</v>
+      </c>
+      <c r="E25">
+        <v>23</v>
+      </c>
+      <c r="F25">
+        <v>0.19491522</v>
+      </c>
+      <c r="G25">
+        <v>0.46597948</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A26">
+        <v>24</v>
+      </c>
+      <c r="B26">
+        <v>0.48</v>
+      </c>
+      <c r="C26">
+        <v>0.44444370999999999</v>
+      </c>
+      <c r="E26">
+        <v>24</v>
+      </c>
+      <c r="F26">
+        <v>0.20338980000000001</v>
+      </c>
+      <c r="G26">
+        <v>0.46521911999999999</v>
+      </c>
+    </row>
+    <row r="27" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A27">
+        <v>25</v>
+      </c>
+      <c r="B27">
+        <v>0.5</v>
+      </c>
+      <c r="C27">
+        <v>0.44250952999999998</v>
+      </c>
+      <c r="E27">
+        <v>25</v>
+      </c>
+      <c r="F27">
+        <v>0.21186437</v>
+      </c>
+      <c r="G27">
+        <v>0.46422855000000002</v>
+      </c>
+    </row>
+    <row r="28" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A28">
+        <v>26</v>
+      </c>
+      <c r="B28">
+        <v>0.52</v>
+      </c>
+      <c r="C28">
+        <v>0.44038599</v>
+      </c>
+      <c r="E28">
+        <v>26</v>
+      </c>
+      <c r="F28">
+        <v>0.22033895000000001</v>
+      </c>
+      <c r="G28">
+        <v>0.46323663999999998</v>
+      </c>
+    </row>
+    <row r="29" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A29">
+        <v>27</v>
+      </c>
+      <c r="B29">
+        <v>0.54</v>
+      </c>
+      <c r="C29">
+        <v>0.43808888000000001</v>
+      </c>
+      <c r="E29">
+        <v>27</v>
+      </c>
+      <c r="F29">
+        <v>0.22881351999999999</v>
+      </c>
+      <c r="G29">
+        <v>0.46196310000000002</v>
+      </c>
+    </row>
+    <row r="30" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A30">
+        <v>28</v>
+      </c>
+      <c r="B30">
+        <v>0.56000000000000005</v>
+      </c>
+      <c r="C30">
+        <v>0.43564523999999999</v>
+      </c>
+      <c r="E30">
+        <v>28</v>
+      </c>
+      <c r="F30">
+        <v>0.2372881</v>
+      </c>
+      <c r="G30">
+        <v>0.46068764000000001</v>
+      </c>
+    </row>
+    <row r="31" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A31">
+        <v>29</v>
+      </c>
+      <c r="B31">
+        <v>0.57999999999999996</v>
+      </c>
+      <c r="C31">
+        <v>0.43316806000000002</v>
+      </c>
+      <c r="E31">
+        <v>29</v>
+      </c>
+      <c r="F31">
+        <v>0.24576268000000001</v>
+      </c>
+      <c r="G31">
+        <v>0.45908892000000001</v>
+      </c>
+    </row>
+    <row r="32" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A32">
+        <v>30</v>
+      </c>
+      <c r="B32">
+        <v>0.6</v>
+      </c>
+      <c r="C32">
+        <v>0.43062085</v>
+      </c>
+      <c r="E32">
+        <v>30</v>
+      </c>
+      <c r="F32">
+        <v>0.25423725000000003</v>
+      </c>
+      <c r="G32">
+        <v>0.45748892000000002</v>
+      </c>
+    </row>
+    <row r="33" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A33">
+        <v>31</v>
+      </c>
+      <c r="B33">
+        <v>0.62</v>
+      </c>
+      <c r="C33">
+        <v>0.42825240999999997</v>
+      </c>
+      <c r="E33">
+        <v>31</v>
+      </c>
+      <c r="F33">
+        <v>0.26271182999999998</v>
+      </c>
+      <c r="G33">
+        <v>0.45574121000000001</v>
+      </c>
+    </row>
+    <row r="34" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A34">
+        <v>32</v>
+      </c>
+      <c r="B34">
+        <v>0.64</v>
+      </c>
+      <c r="C34">
+        <v>0.4265195</v>
+      </c>
+      <c r="E34">
+        <v>32</v>
+      </c>
+      <c r="F34">
+        <v>0.27118639999999999</v>
+      </c>
+      <c r="G34">
+        <v>0.45399355000000002</v>
+      </c>
+    </row>
+    <row r="35" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A35">
+        <v>33</v>
+      </c>
+      <c r="B35">
+        <v>0.66</v>
+      </c>
+      <c r="C35">
+        <v>0.42578650000000001</v>
+      </c>
+      <c r="E35">
+        <v>33</v>
+      </c>
+      <c r="F35">
+        <v>0.27966097000000001</v>
+      </c>
+      <c r="G35">
+        <v>0.45232782999999999</v>
+      </c>
+    </row>
+    <row r="36" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A36">
+        <v>34</v>
+      </c>
+      <c r="B36">
+        <v>0.68</v>
+      </c>
+      <c r="C36">
+        <v>0.42630374999999998</v>
+      </c>
+      <c r="E36">
+        <v>34</v>
+      </c>
+      <c r="F36">
+        <v>0.28813555000000002</v>
+      </c>
+      <c r="G36">
+        <v>0.45066324000000002</v>
+      </c>
+    </row>
+    <row r="37" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A37">
+        <v>35</v>
+      </c>
+      <c r="B37">
+        <v>0.7</v>
+      </c>
+      <c r="C37">
+        <v>0.42816236000000002</v>
+      </c>
+      <c r="E37">
+        <v>35</v>
+      </c>
+      <c r="F37">
+        <v>0.29661013000000003</v>
+      </c>
+      <c r="G37">
+        <v>0.44916756000000002</v>
+      </c>
+    </row>
+    <row r="38" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A38">
+        <v>36</v>
+      </c>
+      <c r="B38">
+        <v>0.72</v>
+      </c>
+      <c r="C38">
+        <v>0.43120671999999999</v>
+      </c>
+      <c r="E38">
+        <v>36</v>
+      </c>
+      <c r="F38">
+        <v>0.30508469999999999</v>
+      </c>
+      <c r="G38">
+        <v>0.44767460999999997</v>
+      </c>
+    </row>
+    <row r="39" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A39">
+        <v>37</v>
+      </c>
+      <c r="B39">
+        <v>0.74</v>
+      </c>
+      <c r="C39">
+        <v>0.43515010999999998</v>
+      </c>
+      <c r="E39">
+        <v>37</v>
+      </c>
+      <c r="F39">
+        <v>0.31355928</v>
+      </c>
+      <c r="G39">
+        <v>0.44623963999999999</v>
+      </c>
+    </row>
+    <row r="40" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A40">
+        <v>38</v>
+      </c>
+      <c r="B40">
+        <v>0.76</v>
+      </c>
+      <c r="C40">
+        <v>0.43985079999999999</v>
+      </c>
+      <c r="E40">
+        <v>38</v>
+      </c>
+      <c r="F40">
+        <v>0.32203385000000001</v>
+      </c>
+      <c r="G40">
+        <v>0.44480872999999999</v>
+      </c>
+    </row>
+    <row r="41" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A41">
+        <v>39</v>
+      </c>
+      <c r="B41">
+        <v>0.78</v>
+      </c>
+      <c r="C41">
+        <v>0.44524525999999998</v>
+      </c>
+      <c r="E41">
+        <v>39</v>
+      </c>
+      <c r="F41">
+        <v>0.33050842000000002</v>
+      </c>
+      <c r="G41">
+        <v>0.44334434</v>
+      </c>
+    </row>
+    <row r="42" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A42">
+        <v>40</v>
+      </c>
+      <c r="B42">
+        <v>0.8</v>
+      </c>
+      <c r="C42">
+        <v>0.45118132</v>
+      </c>
+      <c r="E42">
+        <v>40</v>
+      </c>
+      <c r="F42">
+        <v>0.33898299999999998</v>
+      </c>
+      <c r="G42">
+        <v>0.44188388000000001</v>
+      </c>
+    </row>
+    <row r="43" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A43">
+        <v>41</v>
+      </c>
+      <c r="B43">
+        <v>0.82</v>
+      </c>
+      <c r="C43">
+        <v>0.45747492000000001</v>
+      </c>
+      <c r="E43">
+        <v>41</v>
+      </c>
+      <c r="F43">
+        <v>0.34745757999999999</v>
+      </c>
+      <c r="G43">
+        <v>0.44044678999999998</v>
+      </c>
+    </row>
+    <row r="44" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A44">
+        <v>42</v>
+      </c>
+      <c r="B44">
+        <v>0.84</v>
+      </c>
+      <c r="C44">
+        <v>0.46395199999999998</v>
+      </c>
+      <c r="E44">
+        <v>42</v>
+      </c>
+      <c r="F44">
+        <v>0.35593215</v>
+      </c>
+      <c r="G44">
+        <v>0.43901251000000002</v>
+      </c>
+    </row>
+    <row r="45" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A45">
+        <v>43</v>
+      </c>
+      <c r="B45">
+        <v>0.86</v>
+      </c>
+      <c r="C45">
+        <v>0.47029625000000003</v>
+      </c>
+      <c r="E45">
+        <v>43</v>
+      </c>
+      <c r="F45">
+        <v>0.36440672000000002</v>
+      </c>
+      <c r="G45">
+        <v>0.43771446000000003</v>
+      </c>
+    </row>
+    <row r="46" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A46">
+        <v>44</v>
+      </c>
+      <c r="B46">
+        <v>0.88</v>
+      </c>
+      <c r="C46">
+        <v>0.4761572</v>
+      </c>
+      <c r="E46">
+        <v>44</v>
+      </c>
+      <c r="F46">
+        <v>0.37288130000000003</v>
+      </c>
+      <c r="G46">
+        <v>0.43641889</v>
+      </c>
+    </row>
+    <row r="47" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A47">
+        <v>45</v>
+      </c>
+      <c r="B47">
+        <v>0.9</v>
+      </c>
+      <c r="C47">
+        <v>0.48118638000000002</v>
+      </c>
+      <c r="E47">
+        <v>45</v>
+      </c>
+      <c r="F47">
+        <v>0.38135587999999998</v>
+      </c>
+      <c r="G47">
+        <v>0.43539305</v>
+      </c>
+    </row>
+    <row r="48" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A48">
+        <v>46</v>
+      </c>
+      <c r="B48">
+        <v>0.92</v>
+      </c>
+      <c r="C48">
+        <v>0.48525578000000003</v>
+      </c>
+      <c r="E48">
+        <v>46</v>
+      </c>
+      <c r="F48">
+        <v>0.38983045</v>
+      </c>
+      <c r="G48">
+        <v>0.43436929000000002</v>
+      </c>
+    </row>
+    <row r="49" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A49">
+        <v>47</v>
+      </c>
+      <c r="B49">
+        <v>0.94</v>
+      </c>
+      <c r="C49">
+        <v>0.48792676000000001</v>
+      </c>
+      <c r="E49">
+        <v>47</v>
+      </c>
+      <c r="F49">
+        <v>0.39830502000000001</v>
+      </c>
+      <c r="G49">
+        <v>0.43362592999999999</v>
+      </c>
+    </row>
+    <row r="50" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A50">
+        <v>48</v>
+      </c>
+      <c r="B50">
+        <v>0.96</v>
+      </c>
+      <c r="C50">
+        <v>0.48913962</v>
+      </c>
+      <c r="E50">
+        <v>48</v>
+      </c>
+      <c r="F50">
+        <v>0.40677960000000002</v>
+      </c>
+      <c r="G50">
+        <v>0.43288390999999998</v>
+      </c>
+    </row>
+    <row r="51" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A51">
+        <v>49</v>
+      </c>
+      <c r="B51">
+        <v>0.98</v>
+      </c>
+      <c r="C51">
+        <v>0.48900544000000001</v>
+      </c>
+      <c r="E51">
+        <v>49</v>
+      </c>
+      <c r="F51">
+        <v>0.41525417999999997</v>
+      </c>
+      <c r="G51">
+        <v>0.43222160999999998</v>
+      </c>
+    </row>
+    <row r="52" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A52">
+        <v>50</v>
+      </c>
+      <c r="B52">
+        <v>1</v>
+      </c>
+      <c r="C52">
+        <v>0.48766811999999998</v>
+      </c>
+      <c r="E52">
+        <v>50</v>
+      </c>
+      <c r="F52">
+        <v>0.42372874999999999</v>
+      </c>
+      <c r="G52">
+        <v>0.43155992999999998</v>
+      </c>
+    </row>
+    <row r="53" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="E53">
+        <v>51</v>
+      </c>
+      <c r="F53">
+        <v>0.43220333</v>
+      </c>
+      <c r="G53">
+        <v>0.43091254000000001</v>
+      </c>
+    </row>
+    <row r="54" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="E54">
+        <v>52</v>
+      </c>
+      <c r="F54">
+        <v>0.44067790000000001</v>
+      </c>
+      <c r="G54">
+        <v>0.43026740000000002</v>
+      </c>
+    </row>
+    <row r="55" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="E55">
+        <v>53</v>
+      </c>
+      <c r="F55">
+        <v>0.44915247000000003</v>
+      </c>
+      <c r="G55">
+        <v>0.42978358</v>
+      </c>
+    </row>
+    <row r="56" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="E56">
+        <v>54</v>
+      </c>
+      <c r="F56">
+        <v>0.45762704999999998</v>
+      </c>
+      <c r="G56">
+        <v>0.42930288999999999</v>
+      </c>
+    </row>
+    <row r="57" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="E57">
+        <v>55</v>
+      </c>
+      <c r="F57">
+        <v>0.46610162999999999</v>
+      </c>
+      <c r="G57">
+        <v>0.42906586000000002</v>
+      </c>
+    </row>
+    <row r="58" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="E58">
+        <v>56</v>
+      </c>
+      <c r="F58">
+        <v>0.4745762</v>
+      </c>
+      <c r="G58">
+        <v>0.42882979999999998</v>
+      </c>
+    </row>
+    <row r="59" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="E59">
+        <v>57</v>
+      </c>
+      <c r="F59">
+        <v>0.48305077000000002</v>
+      </c>
+      <c r="G59">
+        <v>0.42864949000000002</v>
+      </c>
+    </row>
+    <row r="60" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="E60">
+        <v>58</v>
+      </c>
+      <c r="F60">
+        <v>0.49152535000000003</v>
+      </c>
+      <c r="G60">
+        <v>0.42846964999999998</v>
+      </c>
+    </row>
+    <row r="61" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="E61">
+        <v>59</v>
+      </c>
+      <c r="F61">
+        <v>0.49999992999999998</v>
+      </c>
+      <c r="G61">
+        <v>0.42820206999999999</v>
+      </c>
+    </row>
+    <row r="62" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="E62">
+        <v>60</v>
+      </c>
+      <c r="F62">
+        <v>0.50847450000000005</v>
+      </c>
+      <c r="G62">
+        <v>0.42793581000000003</v>
+      </c>
+    </row>
+    <row r="63" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="E63">
+        <v>61</v>
+      </c>
+      <c r="F63">
+        <v>0.51694907000000001</v>
+      </c>
+      <c r="G63">
+        <v>0.42771532000000001</v>
+      </c>
+    </row>
+    <row r="64" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="E64">
+        <v>62</v>
+      </c>
+      <c r="F64">
+        <v>0.52542365000000002</v>
+      </c>
+      <c r="G64">
+        <v>0.42749680000000001</v>
+      </c>
+    </row>
+    <row r="65" spans="5:7" x14ac:dyDescent="0.3">
+      <c r="E65">
+        <v>63</v>
+      </c>
+      <c r="F65">
+        <v>0.53389821999999998</v>
+      </c>
+      <c r="G65">
+        <v>0.42745514000000001</v>
+      </c>
+    </row>
+    <row r="66" spans="5:7" x14ac:dyDescent="0.3">
+      <c r="E66">
+        <v>64</v>
+      </c>
+      <c r="F66">
+        <v>0.54237279999999999</v>
+      </c>
+      <c r="G66">
+        <v>0.42741535000000003</v>
+      </c>
+    </row>
+    <row r="67" spans="5:7" x14ac:dyDescent="0.3">
+      <c r="E67">
+        <v>65</v>
+      </c>
+      <c r="F67">
+        <v>0.55084738</v>
+      </c>
+      <c r="G67">
+        <v>0.42759623000000002</v>
+      </c>
+    </row>
+    <row r="68" spans="5:7" x14ac:dyDescent="0.3">
+      <c r="E68">
+        <v>66</v>
+      </c>
+      <c r="F68">
+        <v>0.55932194999999996</v>
+      </c>
+      <c r="G68">
+        <v>0.42777897999999998</v>
+      </c>
+    </row>
+    <row r="69" spans="5:7" x14ac:dyDescent="0.3">
+      <c r="E69">
+        <v>67</v>
+      </c>
+      <c r="F69">
+        <v>0.56779652000000003</v>
+      </c>
+      <c r="G69">
+        <v>0.42811188999999999</v>
+      </c>
+    </row>
+    <row r="70" spans="5:7" x14ac:dyDescent="0.3">
+      <c r="E70">
+        <v>68</v>
+      </c>
+      <c r="F70">
+        <v>0.57627110000000004</v>
+      </c>
+      <c r="G70">
+        <v>0.42844613999999998</v>
+      </c>
+    </row>
+    <row r="71" spans="5:7" x14ac:dyDescent="0.3">
+      <c r="E71">
+        <v>69</v>
+      </c>
+      <c r="F71">
+        <v>0.58474567</v>
+      </c>
+      <c r="G71">
+        <v>0.42887331000000001</v>
+      </c>
+    </row>
+    <row r="72" spans="5:7" x14ac:dyDescent="0.3">
+      <c r="E72">
+        <v>70</v>
+      </c>
+      <c r="F72">
+        <v>0.59322025</v>
+      </c>
+      <c r="G72">
+        <v>0.42930146000000002</v>
+      </c>
+    </row>
+    <row r="73" spans="5:7" x14ac:dyDescent="0.3">
+      <c r="E73">
+        <v>71</v>
+      </c>
+      <c r="F73">
+        <v>0.60169483000000001</v>
+      </c>
+      <c r="G73">
+        <v>0.42975590000000002</v>
+      </c>
+    </row>
+    <row r="74" spans="5:7" x14ac:dyDescent="0.3">
+      <c r="E74">
+        <v>72</v>
+      </c>
+      <c r="F74">
+        <v>0.61016939999999997</v>
+      </c>
+      <c r="G74">
+        <v>0.43021253999999998</v>
+      </c>
+    </row>
+    <row r="75" spans="5:7" x14ac:dyDescent="0.3">
+      <c r="E75">
+        <v>73</v>
+      </c>
+      <c r="F75">
+        <v>0.61864397999999998</v>
+      </c>
+      <c r="G75">
+        <v>0.43070751000000002</v>
+      </c>
+    </row>
+    <row r="76" spans="5:7" x14ac:dyDescent="0.3">
+      <c r="E76">
+        <v>74</v>
+      </c>
+      <c r="F76">
+        <v>0.62711855000000005</v>
+      </c>
+      <c r="G76">
+        <v>0.43120595</v>
+      </c>
+    </row>
+    <row r="77" spans="5:7" x14ac:dyDescent="0.3">
+      <c r="E77">
+        <v>75</v>
+      </c>
+      <c r="F77">
+        <v>0.63559312000000001</v>
+      </c>
+      <c r="G77">
+        <v>0.43181671999999999</v>
+      </c>
+    </row>
+    <row r="78" spans="5:7" x14ac:dyDescent="0.3">
+      <c r="E78">
+        <v>76</v>
+      </c>
+      <c r="F78">
+        <v>0.64406770000000002</v>
+      </c>
+      <c r="G78">
+        <v>0.43243105999999998</v>
+      </c>
+    </row>
+    <row r="79" spans="5:7" x14ac:dyDescent="0.3">
+      <c r="E79">
+        <v>77</v>
+      </c>
+      <c r="F79">
+        <v>0.65254226999999998</v>
+      </c>
+      <c r="G79">
+        <v>0.43321780999999998</v>
+      </c>
+    </row>
+    <row r="80" spans="5:7" x14ac:dyDescent="0.3">
+      <c r="E80">
+        <v>78</v>
+      </c>
+      <c r="F80">
+        <v>0.66101684999999999</v>
+      </c>
+      <c r="G80">
+        <v>0.43400782999999998</v>
+      </c>
+    </row>
+    <row r="81" spans="5:7" x14ac:dyDescent="0.3">
+      <c r="E81">
+        <v>79</v>
+      </c>
+      <c r="F81">
+        <v>0.66949143</v>
+      </c>
+      <c r="G81">
+        <v>0.43502440999999997</v>
+      </c>
+    </row>
+    <row r="82" spans="5:7" x14ac:dyDescent="0.3">
+      <c r="E82">
+        <v>80</v>
+      </c>
+      <c r="F82">
+        <v>0.67796599999999996</v>
+      </c>
+      <c r="G82">
+        <v>0.43604457000000002</v>
+      </c>
+    </row>
+    <row r="83" spans="5:7" x14ac:dyDescent="0.3">
+      <c r="E83">
+        <v>81</v>
+      </c>
+      <c r="F83">
+        <v>0.68644057000000003</v>
+      </c>
+      <c r="G83">
+        <v>0.43732399</v>
+      </c>
+    </row>
+    <row r="84" spans="5:7" x14ac:dyDescent="0.3">
+      <c r="E84">
+        <v>82</v>
+      </c>
+      <c r="F84">
+        <v>0.69491515000000004</v>
+      </c>
+      <c r="G84">
+        <v>0.43860950999999998</v>
+      </c>
+    </row>
+    <row r="85" spans="5:7" x14ac:dyDescent="0.3">
+      <c r="E85">
+        <v>83</v>
+      </c>
+      <c r="F85">
+        <v>0.70338972</v>
+      </c>
+      <c r="G85">
+        <v>0.44013275000000002</v>
+      </c>
+    </row>
+    <row r="86" spans="5:7" x14ac:dyDescent="0.3">
+      <c r="E86">
+        <v>84</v>
+      </c>
+      <c r="F86">
+        <v>0.71186430000000001</v>
+      </c>
+      <c r="G86">
+        <v>0.44166603999999998</v>
+      </c>
+    </row>
+    <row r="87" spans="5:7" x14ac:dyDescent="0.3">
+      <c r="E87">
+        <v>85</v>
+      </c>
+      <c r="F87">
+        <v>0.72033888000000001</v>
+      </c>
+      <c r="G87">
+        <v>0.44328474000000001</v>
+      </c>
+    </row>
+    <row r="88" spans="5:7" x14ac:dyDescent="0.3">
+      <c r="E88">
+        <v>86</v>
+      </c>
+      <c r="F88">
+        <v>0.72881344999999997</v>
+      </c>
+      <c r="G88">
+        <v>0.44491585</v>
+      </c>
+    </row>
+    <row r="89" spans="5:7" x14ac:dyDescent="0.3">
+      <c r="E89">
+        <v>87</v>
+      </c>
+      <c r="F89">
+        <v>0.73728802999999998</v>
+      </c>
+      <c r="G89">
+        <v>0.44649826999999997</v>
+      </c>
+    </row>
+    <row r="90" spans="5:7" x14ac:dyDescent="0.3">
+      <c r="E90">
+        <v>88</v>
+      </c>
+      <c r="F90">
+        <v>0.74576260000000005</v>
+      </c>
+      <c r="G90">
+        <v>0.44809381999999998</v>
+      </c>
+    </row>
+    <row r="91" spans="5:7" x14ac:dyDescent="0.3">
+      <c r="E91">
+        <v>89</v>
+      </c>
+      <c r="F91">
+        <v>0.75423717000000001</v>
+      </c>
+      <c r="G91">
+        <v>0.44960991</v>
+      </c>
+    </row>
+    <row r="92" spans="5:7" x14ac:dyDescent="0.3">
+      <c r="E92">
+        <v>90</v>
+      </c>
+      <c r="F92">
+        <v>0.76271175000000002</v>
+      </c>
+      <c r="G92">
+        <v>0.45113906999999998</v>
+      </c>
+    </row>
+    <row r="93" spans="5:7" x14ac:dyDescent="0.3">
+      <c r="E93">
+        <v>91</v>
+      </c>
+      <c r="F93">
+        <v>0.77118631999999998</v>
+      </c>
+      <c r="G93">
+        <v>0.45259044999999998</v>
+      </c>
+    </row>
+    <row r="94" spans="5:7" x14ac:dyDescent="0.3">
+      <c r="E94">
+        <v>92</v>
+      </c>
+      <c r="F94">
+        <v>0.77966089999999999</v>
+      </c>
+      <c r="G94">
+        <v>0.45405624</v>
+      </c>
+    </row>
+    <row r="95" spans="5:7" x14ac:dyDescent="0.3">
+      <c r="E95">
+        <v>93</v>
+      </c>
+      <c r="F95">
+        <v>0.78813548</v>
+      </c>
+      <c r="G95">
+        <v>0.45540003000000001</v>
+      </c>
+    </row>
+    <row r="96" spans="5:7" x14ac:dyDescent="0.3">
+      <c r="E96">
+        <v>94</v>
+      </c>
+      <c r="F96">
+        <v>0.79661004999999996</v>
+      </c>
+      <c r="G96">
+        <v>0.45676240000000001</v>
+      </c>
+    </row>
+    <row r="97" spans="5:7" x14ac:dyDescent="0.3">
+      <c r="E97">
+        <v>95</v>
+      </c>
+      <c r="F97">
+        <v>0.80508462000000003</v>
+      </c>
+      <c r="G97">
+        <v>0.45801246000000001</v>
+      </c>
+    </row>
+    <row r="98" spans="5:7" x14ac:dyDescent="0.3">
+      <c r="E98">
+        <v>96</v>
+      </c>
+      <c r="F98">
+        <v>0.81355920000000004</v>
+      </c>
+      <c r="G98">
+        <v>0.45928313999999998</v>
+      </c>
+    </row>
+    <row r="99" spans="5:7" x14ac:dyDescent="0.3">
+      <c r="E99">
+        <v>97</v>
+      </c>
+      <c r="F99">
+        <v>0.82203377</v>
+      </c>
+      <c r="G99">
+        <v>0.46052575000000001</v>
+      </c>
+    </row>
+    <row r="100" spans="5:7" x14ac:dyDescent="0.3">
+      <c r="E100">
+        <v>98</v>
+      </c>
+      <c r="F100">
+        <v>0.83050835000000001</v>
+      </c>
+      <c r="G100">
+        <v>0.46178088</v>
+      </c>
+    </row>
+    <row r="101" spans="5:7" x14ac:dyDescent="0.3">
+      <c r="E101">
+        <v>99</v>
+      </c>
+      <c r="F101">
+        <v>0.83898293000000002</v>
+      </c>
+      <c r="G101">
+        <v>0.46308433999999998</v>
+      </c>
+    </row>
+    <row r="102" spans="5:7" x14ac:dyDescent="0.3">
+      <c r="E102">
+        <v>100</v>
+      </c>
+      <c r="F102">
+        <v>0.84745749999999997</v>
+      </c>
+      <c r="G102">
+        <v>0.46438994</v>
+      </c>
+    </row>
+    <row r="103" spans="5:7" x14ac:dyDescent="0.3">
+      <c r="E103">
+        <v>101</v>
+      </c>
+      <c r="F103">
+        <v>0.85593207999999998</v>
+      </c>
+      <c r="G103">
+        <v>0.46582235999999999</v>
+      </c>
+    </row>
+    <row r="104" spans="5:7" x14ac:dyDescent="0.3">
+      <c r="E104">
+        <v>102</v>
+      </c>
+      <c r="F104">
+        <v>0.86440665000000005</v>
+      </c>
+      <c r="G104">
+        <v>0.46725633</v>
+      </c>
+    </row>
+    <row r="105" spans="5:7" x14ac:dyDescent="0.3">
+      <c r="E105">
+        <v>103</v>
+      </c>
+      <c r="F105">
+        <v>0.87288122000000001</v>
+      </c>
+      <c r="G105">
+        <v>0.46882960000000001</v>
+      </c>
+    </row>
+    <row r="106" spans="5:7" x14ac:dyDescent="0.3">
+      <c r="E106">
+        <v>104</v>
+      </c>
+      <c r="F106">
+        <v>0.88135580000000002</v>
+      </c>
+      <c r="G106">
+        <v>0.47040977</v>
+      </c>
+    </row>
+    <row r="107" spans="5:7" x14ac:dyDescent="0.3">
+      <c r="E107">
+        <v>105</v>
+      </c>
+      <c r="F107">
+        <v>0.88983036999999998</v>
+      </c>
+      <c r="G107">
+        <v>0.47194008999999998</v>
+      </c>
+    </row>
+    <row r="108" spans="5:7" x14ac:dyDescent="0.3">
+      <c r="E108">
+        <v>106</v>
+      </c>
+      <c r="F108">
+        <v>0.89830494999999999</v>
+      </c>
+      <c r="G108">
+        <v>0.47348068999999998</v>
+      </c>
+    </row>
+    <row r="109" spans="5:7" x14ac:dyDescent="0.3">
+      <c r="E109">
+        <v>107</v>
+      </c>
+      <c r="F109">
+        <v>0.90677953</v>
+      </c>
+      <c r="G109">
+        <v>0.47464234</v>
+      </c>
+    </row>
+    <row r="110" spans="5:7" x14ac:dyDescent="0.3">
+      <c r="E110">
+        <v>108</v>
+      </c>
+      <c r="F110">
+        <v>0.91525409999999996</v>
+      </c>
+      <c r="G110">
+        <v>0.47581240000000002</v>
+      </c>
+    </row>
+    <row r="111" spans="5:7" x14ac:dyDescent="0.3">
+      <c r="E111">
+        <v>109</v>
+      </c>
+      <c r="F111">
+        <v>0.92372867000000003</v>
+      </c>
+      <c r="G111">
+        <v>0.47638794000000001</v>
+      </c>
+    </row>
+    <row r="112" spans="5:7" x14ac:dyDescent="0.3">
+      <c r="E112">
+        <v>110</v>
+      </c>
+      <c r="F112">
+        <v>0.93220325000000004</v>
+      </c>
+      <c r="G112">
+        <v>0.47696629000000001</v>
+      </c>
+    </row>
+    <row r="113" spans="5:7" x14ac:dyDescent="0.3">
+      <c r="E113">
+        <v>111</v>
+      </c>
+      <c r="F113">
+        <v>0.94067782</v>
+      </c>
+      <c r="G113">
+        <v>0.47702480000000003</v>
+      </c>
+    </row>
+    <row r="114" spans="5:7" x14ac:dyDescent="0.3">
+      <c r="E114">
+        <v>112</v>
+      </c>
+      <c r="F114">
+        <v>0.94915240000000001</v>
+      </c>
+      <c r="G114">
+        <v>0.47708181999999999</v>
+      </c>
+    </row>
+    <row r="115" spans="5:7" x14ac:dyDescent="0.3">
+      <c r="E115">
+        <v>113</v>
+      </c>
+      <c r="F115">
+        <v>0.95762698000000002</v>
+      </c>
+      <c r="G115">
+        <v>0.47682298000000001</v>
+      </c>
+    </row>
+    <row r="116" spans="5:7" x14ac:dyDescent="0.3">
+      <c r="E116">
+        <v>114</v>
+      </c>
+      <c r="F116">
+        <v>0.96610154999999998</v>
+      </c>
+      <c r="G116">
+        <v>0.47656331000000002</v>
+      </c>
+    </row>
+    <row r="117" spans="5:7" x14ac:dyDescent="0.3">
+      <c r="E117">
+        <v>115</v>
+      </c>
+      <c r="F117">
+        <v>0.97457612999999998</v>
+      </c>
+      <c r="G117">
+        <v>0.47612222999999998</v>
+      </c>
+    </row>
+    <row r="118" spans="5:7" x14ac:dyDescent="0.3">
+      <c r="E118">
+        <v>116</v>
+      </c>
+      <c r="F118">
+        <v>0.98305070000000006</v>
+      </c>
+      <c r="G118">
+        <v>0.47568112000000001</v>
+      </c>
+    </row>
+    <row r="119" spans="5:7" x14ac:dyDescent="0.3">
+      <c r="E119">
+        <v>117</v>
+      </c>
+      <c r="F119">
+        <v>0.99152534999999997</v>
+      </c>
+      <c r="G119">
+        <v>0.47500200999999997</v>
+      </c>
+    </row>
+    <row r="120" spans="5:7" x14ac:dyDescent="0.3">
+      <c r="E120">
+        <v>118</v>
+      </c>
+      <c r="F120">
+        <v>1</v>
+      </c>
+      <c r="G120">
+        <v>0.47432417999999998</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
+  <tableParts count="2">
+    <tablePart r:id="rId2"/>
+    <tablePart r:id="rId3"/>
+  </tableParts>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Minor change to excel file
</commit_message>
<xml_diff>
--- a/OpenSim practicle/gait.xlsx
+++ b/OpenSim practicle/gait.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Ideas\Biomechanics\OpenSim practicle\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\USER\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{958AF4DF-B601-4714-B69D-547ECEE03B56}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4774EF0D-811B-4662-8A29-B67E876A41ED}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Knee angle" sheetId="1" r:id="rId1"/>
@@ -2966,7 +2966,7 @@
                   <a:cs typeface="+mn-cs"/>
                 </a:defRPr>
               </a:pPr>
-              <a:endParaRPr lang="en-US"/>
+              <a:endParaRPr lang="en-GB"/>
             </a:p>
           </c:txPr>
         </c:title>
@@ -4523,6 +4523,295 @@
     </xdr:sp>
     <xdr:clientData/>
   </xdr:oneCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>518160</xdr:colOff>
+      <xdr:row>3</xdr:row>
+      <xdr:rowOff>137160</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>14</xdr:col>
+      <xdr:colOff>144780</xdr:colOff>
+      <xdr:row>11</xdr:row>
+      <xdr:rowOff>83820</xdr:rowOff>
+    </xdr:to>
+    <xdr:cxnSp macro="">
+      <xdr:nvCxnSpPr>
+        <xdr:cNvPr id="11" name="Straight Arrow Connector 10">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{87360D6C-7E62-AA03-849C-D76E330061E5}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvCxnSpPr/>
+      </xdr:nvCxnSpPr>
+      <xdr:spPr>
+        <a:xfrm flipH="1">
+          <a:off x="6850380" y="685800"/>
+          <a:ext cx="3284220" cy="1409700"/>
+        </a:xfrm>
+        <a:prstGeom prst="straightConnector1">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:ln>
+          <a:solidFill>
+            <a:srgbClr val="7030A0"/>
+          </a:solidFill>
+          <a:tailEnd type="triangle"/>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </xdr:style>
+    </xdr:cxnSp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>190500</xdr:colOff>
+      <xdr:row>5</xdr:row>
+      <xdr:rowOff>60960</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>14</xdr:col>
+      <xdr:colOff>160020</xdr:colOff>
+      <xdr:row>11</xdr:row>
+      <xdr:rowOff>160020</xdr:rowOff>
+    </xdr:to>
+    <xdr:cxnSp macro="">
+      <xdr:nvCxnSpPr>
+        <xdr:cNvPr id="14" name="Straight Arrow Connector 13">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{1037D50B-4393-0236-4988-D557CBC729B4}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvCxnSpPr/>
+      </xdr:nvCxnSpPr>
+      <xdr:spPr>
+        <a:xfrm flipH="1">
+          <a:off x="8351520" y="975360"/>
+          <a:ext cx="1798320" cy="1196340"/>
+        </a:xfrm>
+        <a:prstGeom prst="straightConnector1">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:ln>
+          <a:solidFill>
+            <a:srgbClr val="7030A0"/>
+          </a:solidFill>
+          <a:tailEnd type="triangle"/>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="1">
+          <a:schemeClr val="accent2"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:schemeClr val="accent2"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="accent2"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </xdr:style>
+    </xdr:cxnSp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>13</xdr:col>
+      <xdr:colOff>594360</xdr:colOff>
+      <xdr:row>2</xdr:row>
+      <xdr:rowOff>83820</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="805220" cy="264560"/>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="15" name="TextBox 14">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{21A39800-90BF-0915-D86A-20ECB35AD159}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr txBox="1"/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="9974580" y="449580"/>
+          <a:ext cx="805220" cy="264560"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="none" rtlCol="0" anchor="t">
+          <a:spAutoFit/>
+        </a:bodyPr>
+        <a:lstStyle/>
+        <a:p>
+          <a:r>
+            <a:rPr lang="en-GB" sz="1100"/>
+            <a:t>Heel Strike</a:t>
+          </a:r>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>14</xdr:col>
+      <xdr:colOff>121920</xdr:colOff>
+      <xdr:row>4</xdr:row>
+      <xdr:rowOff>7620</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="590290" cy="264560"/>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="16" name="TextBox 15">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{3AA3BDD6-5FB9-6B2D-01CF-3B91DD5E4F48}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr txBox="1"/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="10111740" y="739140"/>
+          <a:ext cx="590290" cy="264560"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="none" rtlCol="0" anchor="t">
+          <a:spAutoFit/>
+        </a:bodyPr>
+        <a:lstStyle/>
+        <a:p>
+          <a:r>
+            <a:rPr lang="en-GB" sz="1100"/>
+            <a:t>Toe off</a:t>
+          </a:r>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>22</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>15</xdr:col>
+      <xdr:colOff>495300</xdr:colOff>
+      <xdr:row>36</xdr:row>
+      <xdr:rowOff>22860</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="17" name="Picture 16" descr="heel strike (initial contact), foot flat, mid stance, heel off, toe off, swing phases (acceleration, mid-swing, deceleration)">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{4FA61B73-3F1D-8A6A-28DD-E948544C27A3}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:srcRect/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="6332220" y="4023360"/>
+          <a:ext cx="4762500" cy="2583180"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:extLst>
+          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a14:hiddenFill>
+          </a:ext>
+        </a:extLst>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
 </xdr:wsDr>
 </file>
 

</xml_diff>